<commit_message>
Added data driven test cases
</commit_message>
<xml_diff>
--- a/bdd-behave/testdata/testdata.xlsx
+++ b/bdd-behave/testdata/testdata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agarw\Desktop\wirpo_capstone_project\bdd-behave\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agarw\Desktop\wirpo_capstone_project\bdd-behave\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFCA418-E4EB-45E5-91EC-C4F9BD179995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B4A9A9-E04E-4DB2-BBCB-A7A5850DD39A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5760" yWindow="1536" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,21 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>product</t>
   </si>
   <si>
     <t>Kids T Shirt</t>
-  </si>
-  <si>
-    <t>Boys Jeans</t>
-  </si>
-  <si>
-    <t>Hoodie</t>
-  </si>
-  <si>
-    <t>Casual Shoes</t>
   </si>
 </sst>
 </file>
@@ -384,20 +375,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="A4" s="2"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>